<commit_message>
Keep the full Wikipedia plot/synopsis section in the synopsis column (no sentence cap)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KDL3UhQCv33aSNNrD9AvGk
</commit_message>
<xml_diff>
--- a/data/synopses.xlsx
+++ b/data/synopses.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="synopses" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="full_plot" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="synopses" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="full_plot" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -477,7 +477,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>synopsis (first sentences of plot)</t>
+          <t>synopsis (full plot / synopsis section)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -535,7 +535,13 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Newlyweds Shrek and Princess Fiona return from their honeymoon to find they have been invited by Fiona's parents to a royal ball to celebrate their marriage. Though Shrek is mortified about visiting the kingdom as an ogre, and resents Fiona's parents for locking her in the tower, Fiona convinces him to attend, and they travel to the kingdom of Far Far Away with Donkey in tow and the fairy tale creatures house sitting. They meet Fiona's parents, King Harold and Queen Lillian, who are repulsed to see they are ogres. At dinner, Shrek and Harold get into a heated argument, and afterwards, Fiona encounters Fairy Godmother, a celebrity potions saleswoman who offers to help Fiona but is mortified to see she is married to Shrek.</t>
+          <t>Newlyweds Shrek and Princess Fiona return from their honeymoon to find they have been invited by Fiona's parents to a royal ball to celebrate their marriage. Though Shrek is mortified about visiting the kingdom as an ogre, and resents Fiona's parents for locking her in the tower, Fiona convinces him to attend, and they travel to the kingdom of Far Far Away with Donkey in tow and the fairy tale creatures house sitting. They meet Fiona's parents, King Harold and Queen Lillian, who are repulsed to see they are ogres. At dinner, Shrek and Harold get into a heated argument, and afterwards, Fiona encounters Fairy Godmother, a celebrity potions saleswoman who offers to help Fiona but is mortified to see she is married to Shrek. Shrek worries he is losing Fiona, especially after finding her childhood diary and reading that she was once seemingly infatuated with Prince Charming.
+Harold is secretly reprimanded by Fairy Godmother, who had arranged with Harold for her son—Charming—to be the one to rescue and marry Fiona; she hopes to use the marriage to rule Far Far Away through Charming. She orders Harold to get rid of Shrek or else lose his own happy ending, so Harold hires swashbuckling outlaw and mercenary Puss in Boots to assassinate Shrek.
+Unable to overpower Shrek, Puss reveals that he was paid by Harold and offers to help him in gratitude for having his own life spared. Shrek, Donkey, and Puss meet with Fairy Godmother at her potions factory to find something to help Shrek appeal to Fiona, but she coldly rejects his request, insisting ogres do not deserve happy endings. They retaliate by stealing a potion labeled "Happily Ever After" and accidentally trashing the factory. Shrek and Donkey drink the potion and soon fall asleep. Back in Far Far Away, Fiona notices Shrek is missing and tries to find him, but she too falls asleep.
+The next morning, Shrek and Fiona awaken to find they are now human, and Donkey is a white stallion. To make the change permanent, Shrek must kiss Fiona by midnight. Shrek, Donkey, and Puss return to the castle; however, Fairy Godmother, having discovered the theft, has sent Charming to pose as human Shrek and win Fiona's love. At Fairy Godmother's urging, Shrek leaves the castle, believing that the best way to make Fiona happy is to let her go.
+Fiona is skeptical of Charming; therefore, to ensure the two will wed, Fairy Godmother gives Harold a love potion to put into Fiona's tea. This exchange is overheard by Shrek, Donkey, and Puss, who are arrested by the royal knights after Donkey inadvertently exposes them. While the ball begins, the fairy tale creatures - having seen the arrest on the news - rescue the trio from the dungeon. They all storm the castle with the help of Mongo, a monstrous living gingerbread man created by the Muffin Man.
+Though Mongo is destroyed, the group manages to break into the ball. Shrek fails to prevent Charming from kissing Fiona, but instead of falling in love, Fiona knocks him out. Harold reveals that he swapped Fiona's tainted teacup with his own, refusing to go through with the plot. Livid, the Fairy Godmother tries to strike Shrek with a spell from her magic wand. Harold jumps in front of it and is struck; the rest of the spell reflects off his breastplate and hits the Fairy Godmother, causing her to disintegrate into bubbles.
+Harold reverts to his true form as the Frog Prince, having used the "Happily Ever After" potion years earlier to gain Lillian's love. He approves of Shrek and Fiona's marriage, while Lillian assures Harold that she still loves him. As the clock strikes midnight, Fiona declines Shrek's offer to remain human, and they revert to ogres, while Donkey also returns to normal, much to his sadness. Everyone celebrates as the ball continues. In a mid-credits scene, Dragon, who had recently married Donkey, arrives with several dragon-donkey hybrid babies.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -583,7 +589,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>In the near future, humanity faces extinction due to dust storms and widespread crop blights. Joseph Cooper, a widowed former NASA test pilot, works as a farmer and raises his children, Murphy "Murph" and Tom, with his father-in-law Donald. Following a dust storm, Cooper and Murph discover that dust patterns in Murph's room, which she had attributed to a ghost, result from a gravitational anomaly. Cooper recognizes the patterns as binary code specifying coordinates, which lead him and Murph to a secret NASA facility headed by Professor John Brand.</t>
+          <t>In the near future, humanity faces extinction due to dust storms and widespread crop blights. Joseph Cooper, a widowed former NASA test pilot, works as a farmer and raises his children, Murphy "Murph" and Tom, with his father-in-law Donald. Following a dust storm, Cooper and Murph discover that dust patterns in Murph's room, which she had attributed to a ghost, result from a gravitational anomaly. Cooper recognizes the patterns as binary code specifying coordinates, which lead him and Murph to a secret NASA facility headed by Professor John Brand.
+Brand explains that 48 years earlier, a wormhole appeared near Saturn, apparently placed there by an unknown intelligence, leading to a system in another galaxy with 12 potentially habitable planets located near a black hole named Gargantua. Volunteers of the Lazarus expedition had previously traveled through the wormhole to evaluate the planets, with three—Miller, Mann, and Edmunds—reporting back desirable results.
+Cooper is enlisted to pilot the Endurance spacecraft through the wormhole as part of a mission to colonize a habitable planet with 5,000 frozen embryos and ensure humanity's survival. Meanwhile, Professor Brand would continue his work on solving a gravity equation whose solution would enable construction of a spacecraft for an exodus from Earth. Cooper accepts against Murph's wishes and promises to return. When she refuses to see him off, he leaves her his wristwatch to compare their relative time when he returns.
+The crew, consisting of Cooper, robots TARS and CASE, and scientists Amelia Brand (Professor Brand's daughter), Romilly, and Doyle, traverses the wormhole after a two-year voyage to Saturn. Cooper, Doyle, and Brand use a lander to investigate Miller's planet, where time is severely dilated. They land in knee-high water and find only wreckage from Miller's expedition before a gigantic tidal wave kills Doyle and waterlogs the lander's engines.
+By the time they leave the planet, Cooper and Brand discover that 23 years have elapsed on the Endurance. Having enough fuel left for only one of the remaining planets, Cooper and Romilly decide to go to Mann's planet, despite Brand's protests, as he is still broadcasting. En route, they receive messages from Earth. Cooper watches Tom grow up, marry, and have his first son, who soon passes away, while an adult Murph is now a scientist working on the gravity equation with Professor Brand. On his deathbed, Professor Brand confesses to Murph that the Endurance crew was never meant to return, since a complete solution to the equation was impossible to obtain without measurements from inside a black hole.
+On Mann's planet, they awaken him from cryostasis, and he assures them that colonization is possible, despite the extreme environment. During a scouting mission, Mann attempts to kill Cooper and reveals that he falsified his data in the hope of being rescued. He steals Cooper's lander and heads for the Endurance. A booby trap set by Mann kills Romilly, but Brand rescues Cooper with the other lander and they race back to the Endurance. Mann is killed in a failed manual docking operation, badly damaging the Endurance, but Cooper is able to regain control of the spacecraft through his own docking maneuver.
+With insufficient fuel, Cooper and Brand resort to a slingshot around Gargantua, which costs them 51 years due to time dilation. In the process, Cooper and TARS detach in their craft to lighten the Endurance so that Brand and CASE may reach Edmunds' planet. Falling past Gargantua's event horizon, they eject from their craft and find themselves in a tesseract made up of infinite copies of Murph's bedroom across moments in time. Cooper deduces that the tesseract was constructed by advanced humans in the far future, and realizes that he had always been Murph's "ghost". Using Morse code, he manipulates the second hand of her wristwatch to transmit the data TARS collected, enabling Murph to complete the gravity equation's solution.
+The tesseract, its purpose fulfilled, collapses, ejecting Cooper and TARS. Cooper wakes up on a station orbiting Saturn. He reunites with Murph, now elderly and on her deathbed, who tells him to seek out Brand. Cooper and TARS take a spacecraft to rejoin Brand and CASE, who are establishing the human colony on Edmunds' planet.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -631,7 +644,13 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>An armed conflict forces young couple Pedro and Alma Madrigal to flee their home village in Colombia with their infant triplets, Julieta, Pepa, and Bruno. Pedro is killed, but the candle Alma carries gains a magical power that repels the attackers and creates Casita, a sentient house located in a magical realm bordered by mountains. Fifty years later, a new village thrives under the candle's protection, which grants "gifts" to each Madrigal descendant when they turn five, which they use to serve the villagers. Bruno, who was vilified and scapegoated for his precognition, disappeared ten years earlier, and Julieta's youngest daughter, Mirabel, inexplicably did not receive a gift.</t>
+          <t>An armed conflict forces young couple Pedro and Alma Madrigal to flee their home village in Colombia with their infant triplets, Julieta, Pepa, and Bruno. Pedro is killed, but the candle Alma carries gains a magical power that repels the attackers and creates Casita, a sentient house located in a magical realm bordered by mountains. 
+Fifty years later, a new village thrives under the candle's protection, which grants "gifts" to each Madrigal descendant when they turn five, which they use to serve the villagers. Bruno, who was vilified and scapegoated for his precognition, disappeared ten years earlier, and Julieta's youngest daughter, Mirabel, inexplicably did not receive a gift.
+On his fifth birthday, Pepa's youngest son, Antonio, is granted the ability to communicate with animals. During the celebration, the Madrigals unwittingly exclude Mirabel from being in a family photo. Mirabel sees Casita cracking and the candle's flame flickering and alerts her family, but Casita repairs itself, causing disbelief in Mirabel. After overhearing Alma lament the candle's fading that night, Mirabel resolves to restore Casita's magic herself. Her older sister Luisa, who possesses superhuman strength, confesses to Mirabel that she feels overwhelmed by her constant obligation to help the villagers using her strength, which has been faltering. She suggests to Mirabel that Bruno's room, located inside a forbidden tower in Casita, may hold the secret to the fading magic.
+Mirabel finds a cave in Bruno's room that holds pieces of his last vision made of opaque emerald. Alma and the family warn Mirabel not to investigate further, but she reassembles the pieces and sees herself with Casita cracking behind her. Mirabel's father Agustín accidentally discovers Mirabel and warns her to keep the vision a secret, but they are overheard by Pepa's daughter Dolores, who possesses supernatural hearing. Mirabel's oldest sister Isabela, who can make plants and flowers instantly grow at will, is scheduled to be engaged to the Madrigals' neighbor Mariano Guzmán. Amidst Mariano's proposal, an awkward dinner, and Dolores telling everyone about Mirabel's discovery, Casita begins to crack again, and everyone loses control of their gifts.
+Mirabel follows rats carrying the pieces of the vision to a secret passage behind a portrait, where she finds Bruno, who reveals he never left Casita, and his visions alternate between Mirabel saving Casita and destroying it, leading him to believe she is the key to the fate of Casita's magic. Not wanting Mirabel to be hurt, he destroyed the vision and isolated himself. At Mirabel's insistence, Bruno conjures another vision that depicts Mirabel and Isabela, who have a strained relationship, hugging, which strengthens the candle.
+Mirabel attempts to apologize to a frustrated Isabela, who confesses she is burdened by her image of perfection and does not want to marry Mariano. Mirabel helps Isabela use her powers more freely and they hug. Alma arrives and angrily blames Mirabel for causing the family's misfortunes out of spite for not having a gift. Mirabel gets into an argument with Alma's behavior and asserts that her harmful expectations for her family are the true cause of Casita dying, which horrifies Alma. In the ensuing argument, Casita is destroyed by the cracks as Mirabel tries to save the candle, which extinguishes in her hands, leaving the Madrigals powerless. Distraught and heartbroken, Mirabel runs away from home.
+The next day, Alma finds Mirabel tearfully sitting beside the river where Pedro was killed by the soldiers and where the miracle had begun. Alma realizes that her obsession with preserving the magic made her oblivious to how her expectations and pressure were harming the family. She expresses remorse, reconciles with Mirabel, and reunites with Bruno. The three return to the village and assemble the other Madrigals to rebuild Casita, and the townspeople join in, restoring the family's gifts and reviving Casita. The Madrigals celebrate and take another family photo, this time including Mirabel and Bruno.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -679,7 +698,14 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Twenty-two years after the Jurassic Park disaster on Isla Nublar in 1993, a new dinosaur theme park called Jurassic World has been built on the island, owned by Masrani Global Corporation in affiliation with InGen, which created the dinosaurs. Brothers Zach and Gray Mitchell visit the park, where their aunt Claire Dearing works as the operations manager. She assigns her assistant Zara to guide them, but they evade her and explore on their own. Navy veteran and ethologist Owen Grady has been training a Velociraptor squad composed of Blue, Charlie, Delta, and Echo, and researching their intelligence.</t>
+          <t>Twenty-two years after the Jurassic Park disaster on Isla Nublar in 1993, a new dinosaur theme park called Jurassic World has been built on the island, owned by Masrani Global Corporation in affiliation with InGen, which created the dinosaurs. Brothers Zach and Gray Mitchell visit the park, where their aunt Claire Dearing works as the operations manager. She assigns her assistant Zara to guide them, but they evade her and explore on their own.
+Navy veteran and ethologist Owen Grady has been training a Velociraptor squad composed of Blue, Charlie, Delta, and Echo, and researching their intelligence. Based on the raptors' ability to follow commands, the head of InGen security Vic Hoskins believes that the animals can be weaponized, an idea Owen and his assistant Barry vehemently oppose.
+Claire and Jurassic World owner Simon Masrani inspect the park's newest upcoming attraction, the Indominus rex, a transgenic dinosaur created by geneticist Dr. Henry Wu. Masrani tasks Owen with evaluating the enclosure's security. Owen warns Claire that the Indominus lacks social skills, making it dangerous and unpredictable. When the Indominus seemingly escapes, Owen and two other workers investigate. The dinosaur, capable of camouflaging itself and masking its heat signature, suddenly appears and devours the other two men, but Owen manages to survive. The Indominus escapes its paddock and into the island's interior. Owen urges Masrani to destroy it, but Masrani, trying to protect his company's investment, sends a unit to subdue it using non-lethal weaponry. After most of the unit is killed, Claire orders the evacuation of the northern sector, while Masrani confronts Wu about the Indominus design.
+While exploring the park in a tour vehicle, Zach and Gray enter a restricted area. The Indominus arrives and destroys the vehicle, but the boys narrowly escape. They find the ruins of the original Jurassic Park visitor center, repair an old Jeep Wrangler, and drive back to the park resort.
+As Claire and Owen search for the boys, they barely escape the Indominus as well. Masrani and two soldiers hunt the Indominus by helicopter, but it breaks into the park's aviary. The Pteranodons and Dimorphodons, startled by the Indominus, flee the aviary and fly into Masrani's helicopter, causing it to crash and kill its passengers. The escaped pterosaurs converge on the resort and attack everyone, including Zara, who is then devoured by a Mosasaurus. Zach and Gray find Owen and Claire at the resort as armed personnel shoot down the pterosaurs.
+Hoskins assumes command and orders the raptors to be used to track the Indominus, whereupon Owen reluctantly complies and spearheads the assault with the raptors. Upon finding it, the dinosaurs begin communicating with one another. Owen realizes that the Indominus has Velociraptor DNA, and it usurps Owen's command of the raptors, becoming the pack's new alpha. Soldiers fire on the Indominus, but it escapes. The raptors slaughter most of the soldiers, while Charlie is killed in the chaos. Hoskins evacuates Wu and the dinosaur embryos from the island to protect his research. Owen, Claire, and the boys find Hoskins at the lab securing more embryos, but Delta breaks in and kills him.
+Owen restores his bond with the three surviving raptors before the Indominus reappears. The raptors attack the hybrid, but Delta and Echo are killed while Blue is knocked unconscious. Claire releases Jurassic Park’s veteran Tyrannosaurus rex  from its paddock and lures it to the Indominus. The dinosaurs attack each other, and the Indominus eventually overpowers the Tyrannosaurus, but Blue recovers and joins the battle. The duo fights the Indominus until it gets cornered at the lagoon's edge, where it is dragged underwater by the Mosasaurus. Owen and Blue part ways afterwards.
+The survivors are evacuated, and the island is abandoned once again. Zach and Gray reunite with their parents, while Owen and Claire decide to stay together.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -727,7 +753,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Three years after becoming a chieftess and wayfinder for her people, Moana spends her days exploring other islands near her home island of Motunui in the hope of finding people connected to the ocean. On her return from one such voyage, Moana is named Motunui's first tautai (master wayfinder) in a thousand years. In a vision, Moana's ancestor, Tautai Vasa, reveals why none of those people are connected anymore: the malicious storm god Nalo wanted power over the mortals, so he sunk a legendary island called Motufetu, which connected all of the islands, down to the depths of the ocean. Vasa further warns that the people of Motunui will go extinct in the future if Moana cannot find a way to raise Motufetu.</t>
+          <t>Three years after becoming a chieftess and wayfinder for her people, Moana spends her days exploring other islands near her home island of Motunui in the hope of finding people connected to the ocean. On her return from one such voyage, Moana is named Motunui's first tautai (master wayfinder) in a thousand years.
+In a vision, Moana's ancestor, Tautai Vasa, reveals why none of those people are connected anymore: the malicious storm god Nalo wanted power over the mortals, so he sunk a legendary island called Motufetu, which connected all of the islands, down to the depths of the ocean. Vasa further warns that the people of Motunui will go extinct in the future if Moana cannot find a way to raise Motufetu. In response to this call from the ancestors, Moana assembles a crew of people from Motunui — craftswoman Loto, historian Moni, and grumpy elderly farmer Kele, alongside her pet pig and rooster, Pua and Heihei — to follow the path of a comet across the ocean towards Motufetu.
+Meanwhile, Maui is seeking Motufetu himself since he had a previous quarrel with Nalo, but he is captured by Nalo's enforcer, Matangi. Maui is reluctant to contact Moana, as he fears she may not survive if she comes to help. Moana and her crew are captured by the Kakamora, a tribe of savage coconut-like pirates that Moana previously encountered, who reveal that Nalo's actions against Motufetu had caused them to be disconnected from their home island. A Kakamora named Kotu helps the crew paralyze a gargantuan monster clam inside of which is Matangi's lair. While the crew finds Maui, Moana meets Matangi and learns that she is not happy serving Nalo. Matangi helps Moana escape and reunite with Maui and her friends, before sending them to where Nalo is.
+Maui warns that Nalo's realm is deadlier compared to the mortal realm and that fighting him will spell certain death for mere mortals. Nalo's monsters ambush the group, damaging their raft and washing them ashore on an isolated island. Moana begins to despair, but Maui encourages her to keep on going. With Moana revitalized, the group plans to have Maui raise Motufetu so that Moana can touch it, as that is the only way to stop Nalo. Her crew repairs her raft, but when the group ventures forth to confront Nalo, they encounter a gigantic storm.
+Moana, realizing that Nalo is trying to stop humans from breaking the curse, asks Maui to lift Motufetu enough for her to touch it. Maui begins to pull up Motufetu with his giant hook, but Nalo strips Maui of his demigod powers with a lightning bolt. Moana, in a moment of desperation, dives into the ocean to touch Motufetu underwater, but as she succeeds, Nalo's lightning kills her. Maui jumps in after her body, and with a magical chant, summons the spirits of Tautai Vasa and Moana's ancestors, including her grandmother Tala, who help revive her as a demigoddess, with Moana gaining a wayfinder's tattoo. Maui, also regaining his powers as a demigod, finally raises Motufetu and helps Moana reconnect the people with the ocean.
+The crew returns home to Motunui, leading a flotilla of the people of the ocean, and a celebration is held in Moana's honor. Meanwhile, Nalo plans his revenge and is about to punish Matangi for helping Moana, when the giant crab Tamatoa arrives to join his cause.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -775,7 +806,13 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Jiang Ziya and Ji Fa gather civilians with the Kunlun immortals to defend Xiqi from the Shang dynasty army. The body of Yin Jiao—former crown prince of the Shang dynasty—is brought to Kunlun by Nezha and Yang Jian to be resurrected. Despite protests that resurrection will go against natural order, The Great Saint decides to resurrect Jiao. However, he finds that Jiao's soul is filled with hatred and vengeance against his father Yin Shou, causing him to absorb the Great Saint's power.</t>
+          <t>Jiang Ziya and Ji Fa gather civilians with the Kunlun immortals to defend Xiqi from the Shang dynasty army. The body of Yin Jiao—former crown prince of the Shang dynasty—is brought to Kunlun by Nezha and Yang Jian to be resurrected. Despite protests that resurrection will go against natural order, The Great Saint decides to resurrect Jiao. However, he finds that Jiao's soul is filled with hatred and vengeance against his father Yin Shou, causing him to absorb the Great Saint's power.
+King Yin Shou, newly resurrected by the fox spirit, welcomes Grand Preceptor Wen Zhong and his armies home to Zhaoge after 10 years at war, alongside his generals Deng Chanyu and the Four Demonic Giants. They welcome Shou in the palace, who requests Zhong to capture Ji Fa and Ziya for the Investiture Scroll. Zhong declines and seeks retirement after a long hardship of protecting their dynasty but Chanyu requests to lead the mission, honoring her late father's wishes for her to become a renowned warrior.
+Shou sends an emissary, ordering Ji Fa to commit suicide or risk an invasion of Xiqi, which Ji Fa refuses. Though his troops manage to fend off Chanyu's forces, they were overpowered and hastily retreat. Chanyu pursues Ji Fa, who barely escapes. Ji Fa reunites with Ziya who was captured by Shen Gongbao's crows, confessing that he ordered Xiqi's evacuation. Ziya then convinces him to continue fighting against Shou. Meanwhile, the fox spirit, severely weakened trying to restore Shou to full health, is unable to keep Daji's body fresh anymore. They search for a new vessel for the spirit, only to find that she is unable to leave Daji's body.
+Upon Ji Fa and Ziya's return, Ziya suggests Ji Fa's forces to attack Chanyu's encampment later that night. Though they managed to kill one of the giants at Chanyu's camp, they were unable to defeat the remainder who assault the city the following day. Jiao, having absorbed the Great Saint's power, kills the remaining giants while Ji Fa rescues Chanyu from drowning and offers to surrender in exchange for Chanyu's forces sparing Xiqi and its inhabitants. Meanwhile, Shou coerces Zhong to reassume command of his forces.
+Chanyu brings Ji Fa to Zhong, who refuses Ji Fa's plea to surrender and orders a massacre on Xiqi. Disgusted by Zhong's willingness to kill innocents, Chanyu helps Ji Fa escape imprisonment. Zhong pursues them, but Jiao holds him back, swearing to kill him if the invasion continues. Jiao reunites with Ji Fa, and Chanyu is accepted as a guest in Xiqi for saving Ji Fa, while the Tongtian Cult Leader grants Gongbao a gourd of Gu to kill Shou's remaining forces and resurrect them as obedient, undead soldiers.
+Zhong cloaks Xiqi in darkness and summons floating mirrors that incapacitate anyone caught in their beams in a ritual; Chanyu's forces—now under Zhong's command—are protected by a sigil, allowing them to breach the city unimpeded, which Ziya recognises from a similar mark on Chanyu. Ziya realizes that Zhong is after him and the Scroll; Chanyu bargained with Zhong to bring Ziya and the Scroll in exchange for sparing Xiqi, allowing himself to be captured by Chanyu and brought to Zhong's altar. Ziya indicates Zhong's location to Ji Fa with a flare.
+At the altar, Ji Fa prepares to kill Zhong as he completes the ritual to wipe out everyone affected by his mirrors; conversely, this will also eliminate everyone protected by his sigil—including Chanyu. After defeating Zhong's qilin, Chanyu helps Ji Fa kill Zhong, stopping the ritual and returning Ji Fa's allies to consciousness as Zhong's troops and Chanyu dissipate. Jiao travels alone back to Zhaoge to kill Shou, but is halted by the Tongtian Leader; Gongbao meets Zhong to collect his head according to the King's orders, leading an army of Gu soldiers onto Xiqi. The Tongtian Leader raises a brainwashed Jiao from a pool of mercury, presenting him to Shou and Daji as their puppet.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -823,7 +860,13 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>In 1969, Iris Campbell and her boyfriend Paul attend the grand opening of the Sky View, an observation tower restaurant. Iris has a premonition that a chain of events will cause the tower to collapse, killing everyone inside. She warns the attendees and prevents the disaster, but in doing so disrupts Death's design. Fifty-five years later, Iris and Paul's granddaughter, college student Stefani Reyes, is plagued by recurring nightmares of the averted disaster and returns home seeking answers.</t>
+          <t>In 1969, Iris Campbell and her boyfriend Paul attend the grand opening of the Sky View, an observation tower restaurant. Iris has a premonition that a chain of events will cause the tower to collapse, killing everyone inside. She warns the attendees and prevents the disaster, but in doing so disrupts Death's design.
+Fifty-five years later, Iris and Paul's granddaughter, college student Stefani Reyes, is plagued by recurring nightmares of the averted disaster and returns home seeking answers. She reunites with her father, Marty, and younger brother Charlie, then visits her uncle Howard, aunt Brenda, and cousins Erik, Julia, and Bobby. When Stefani asks about Iris, Howard explains that he and Stefani's mother, Darlene, were raised in an overprotective, isolated environment, contributing to family tensions and Darlene's absence. Brenda helps Stefani find letters from Iris leading to a fortified cabin where Iris, terminally ill with cancer, now lives.
+Iris recounts the Sky View incident, explaining that after she prevented the collapse, Death began killing the survivors in the order they were originally meant to die, along with their descendants. Following Paul's death, Iris documented Death's actions in a notebook to protect her family. Stefani doubts her story and tries to leave, but Iris follows her outside, gives her the notebook, and allows herself to be fatally impaled by a weather vane to prove her claims.
+At Iris's funeral, Darlene returns, but Stefani resents her for abandoning her and Charlie during their childhood. The notebook mentions "JB", who discovered someone who defeated Death. During a family barbecue, a chain of events kills Howard with his lawnmower. After his funeral, Stefani warns the family that Death is coming, but they remain skeptical. A fire breaks out at Erik's tattoo shop, but his leather jacket saves him. The next day, Stefani and Charlie try to protect Erik, believing he is next, but Julia is crushed by a garbage truck's compactor. Brenda then reveals that Erik was the product of an affair and is not part of Iris's bloodline, explaining why he was spared.
+Darlene suggests finding "JB", who is William Bludworth. A child at the Sky View and the final person to die in Iris's original premonition, Bludworth explains that Iris later found him and that they learned Death's rules together. He tells the family that Death can be defeated either by taking another life or by becoming clinically dead and then being resuscitated, citing Kimberly Corman as an example. Bludworth leaves, expecting his cancer to kill him once Iris's bloodline ends.
+Erik persuades Bobby to use the second method by triggering a fatal allergic reaction to nuts and then reviving him. The plan fails when a malfunctioning MRI machine tears out Erik's piercings and pulls him inside; a wheelchair then impales and crushes him, while a vending-machine coil launches into Bobby's head. Stefani, Charlie, and Darlene flee to Iris's cabin, hoping to hide Darlene from Death. They crash through the front gate, Stefani's seat belt jams, and the cabin explodes, sending Darlene's RV into the water with Stefani trapped inside. Darlene saves Charlie before being crushed by a lamp post, while Charlie rescues and resuscitates Stefani.
+One week later, the father of Charlie's prom date, a physician, explains that Stefani was never clinically dead because she was resuscitated before cardiac arrest. Moments later, a timber-carrying freight train derails nearby, and its cargo fatally crushes the siblings.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -871,7 +914,9 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>John, a single dad to four year old son Michael, has received a terminal cancer diagnosis. In his final exercise of urgency, the father must choose a new adoptive household for his son, as Michael's mother left them when Michael was 6 months old. To do this, he is forced to participate in a series of auditions; various potential parental pairs offer themselves, but simultaneously reveal themselves as repulsive or unsuitable. A woman, living alone, is the exception.</t>
+          <t>John, a single dad to four year old son Michael, has received a terminal cancer diagnosis. In his final exercise of urgency, the father must choose a new adoptive household for his son, as Michael's mother left them when Michael was 6 months old.  To do this, he is forced to participate in a series of auditions; various potential parental pairs offer themselves, but simultaneously reveal themselves as repulsive or unsuitable. A woman, living alone, is the exception. She depicts herself as troubled, but honest about herself and her identity. She got pregnant as a teen and was forced to give her child up for adoption. Later when she married and wanted children with her husband, she was informed by doctors that she wouldn't be able to have any biological children. The woman was open to adoption but her husband was not, feeling he couldn't love a child that wasn't biologically his, so they separated.
+John is reluctant to explain that he will be dying to Michael, fearing it would be too much for the young boy to handle. John's acquaintances are sympathetic to his situation and his social workers are eager for him to make a decision, but he hesitates as it will be the biggest decision he'll ever make, and he wants Michael to have the life and opportunities he never did.
+Soon John's illness progresses and he has to give up his job as a window cleaner. Michael observes John's deterioration, witnessing him sleep a lot and have weak moments such as struggling to pour his orange juice. John finally explains the situation to Michael, and explains that though Michael won't be able to hear him physically, he'll be able to hear him inside in his heart. John puts together a memory box with letters for Michael to read when he reaches certain milestones, John's window cleaning tools, pictures taken at a fair ground, and a picture of Michael being held by his birth mum inside the young woman's glove that John found when cleaning out his light truck to sell. In the final minutes of the film John and Michael reveal that they have chosen the single mum as Michael's future parent.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -919,7 +964,14 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>After Ne Zha and Ao Bing are struck by godly lightning together, their bodies are destroyed. To prevent their souls from dying, Master Taiyi Zhenren exhausts his Seven-Colored Sacred Lotus to regenerate their physical bodies, though they are still fragile. Ao Bing's father Ao Guang, the Dragon King of the East Sea, believing his son is dead, orders Master Shen Gongbao to attack Chentang Pass with the demons imprisoned under his palace and the other three Dragon Kings of the Four Seas. Ao Bing defends Chentang Pass, but his new body disintegrates due to the effort exerted.</t>
+          <t>After Ne Zha and Ao Bing are struck by godly lightning together, their bodies are destroyed. To prevent their souls from dying, Master Taiyi Zhenren exhausts his Seven-Colored Sacred Lotus to regenerate their physical bodies, though they are still fragile. Ao Bing's father Ao Guang, the Dragon King of the East Sea, believing his son is dead, orders Master Shen Gongbao to attack Chentang Pass with the demons imprisoned under his palace and the other three Dragon Kings of the Four Seas. Ao Bing defends Chentang Pass, but his new body disintegrates due to the effort exerted.
+Ao Guang makes a ceasefire deal: Ao Bing and Ne Zha will share Ne Zha's body for seven days, complete three trials to become a xian (immortal) and win a potion that can restore the Sacred Lotus and create a new body for Ao Bing, upon which Ao Guang's forces will retreat. The trials are set by Immortal Wuliang, leader of the heavenly Chan sect. During the trials, candidates complete missions, which were normally performed by the sect's demon hunters, while supervised by Wuliang's disciples Deero and Crana.
+Ne Zha takes sleeping pills to hide his demon nature during the trials, allowing Ao Bing to fully control his body temporarily. Together, Ne Zha and Ao Bing complete the first two trials: defeating a village of marmot demons and a master who trains demons to prepare for the xian trials, respectively.
+In the meantime, Ao Guang tasks Shen Gongbao with guarding the Chentang Pass. Gongbao is temporarily reunited with his younger brother Shen Xiaobao. Xiaobao then witnesses Ne Zha's second trial where the master Shen Zhengdao, the Shen family's patriarch, is violently captured by the sect's forces. He returns to tell Gongbao of the sect's siege and plunder of their family's village, but is fatally wounded by Deero, dying from his injuries.
+Before Ne Zha sets off on his third trial, he is informed that Chentang Pass was destroyed. Enraged, Ne Zha completes the third trial without Ao Bing's help, defeating the stone spirit Shi Ji, becoming xian and obtaining the potion. While Taiyi restores the Sacred Lotus with the potion and regenerates Ao Bing's body, Ne Zha joins Wuliang's forces to trap the dragons in Wuliang's giant cauldron, planning to forge the dragons and demons into Pills of Immortality. However, the other three dragon kings turn against Ao Guang by collaborating with Wuliang to escape the cauldron.
+However, Li Jing and Lady Yin arrive at the cauldron unharmed with Ao Bing and Taiyi to explain the truth: Wuliang ordered the destruction of Chentang Pass and framed the dragons for it; he even convinced the other dragon kings to betray Ao Guang and frame him for the attack, all part of Wuliang's true plot to ensure the heavenly sect's domination. Nezha's parents escaped the destruction while Shen, who knew the truth of the attack, took a last stand to defend the city.
+Exposed, Wuliang casts Ne Zha's group into the cauldron. As the heat of the cauldron rises, the prisoners are transformed into Pills of Immortality, including Lady Yin. A grieving Ne Zha absorbs the cauldron's samadhi fire, solidifying his new body, and thus is reborn. Alongside the dragons and demons, Ne Zha and Ao Bing break the cauldron and force Wuliang and his cohorts to retreat. In the aftermath, Ao Guang leads the remaining dragons and demons into hiding in the seas while allowing Ao Bing to stay behind and help Ne Zha expose Wuliang's nature.
+Wuliang, Deero, and Crana head to a secret prison where Wuliang negotiates with the captive Shen Gongbao and Shen Zhengdao, hoping to recruit them, only to be trapped after Wuliang cursed a warden to sleep for 10 years for mocking his injuries, and that his registered injuries have healed. Ne Zha's older xian brothers Jinzha and Muzha are summoned to meet with Wuliang, but cannot find him when they arrive. Deero and Crana work to get Wuliang's injuries back to match the registered picture.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -967,7 +1019,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>After being rescued by the Fingers, a gang led by the psychopathic Satan worshipper, "Sir Lord" Jimmy Crystal, Spike is forced to kill Jimmy Shite in a death match, as an initiation. Sir Jimmy then renames the young boy "Jimmy" to match the other Fingers, who include the slightly empathetic Jimmy Ink, and the deranged, sadistic Jimmima. Dr Ian Kelson, who covers his skin in iodine solution to protect himself from the virus, continues to build up the Bone Temple, an ossuary for those killed in the Rage Virus epidemic, while the Alpha Infected, Samson, repeatedly visits him. Kelson deduces that Samson is becoming addicted to the morphine from his blowgun, deliberately allowing himself to be drugged.</t>
+          <t>After being rescued by the Fingers, a gang led by the psychopathic Satan worshipper, "Sir Lord" Jimmy Crystal, Spike is forced to kill Jimmy Shite in a death match, as an initiation. Sir Jimmy then renames the young boy "Jimmy" to match the other Fingers, who include the slightly empathetic Jimmy Ink, and the deranged, sadistic Jimmima.
+Dr Ian Kelson, who covers his skin in iodine solution to protect himself from the virus, continues to build up the Bone Temple, an ossuary for those killed in the Rage Virus epidemic, while the Alpha Infected, Samson, repeatedly visits him. Kelson deduces that Samson is becoming addicted to the morphine from his blowgun, deliberately allowing himself to be drugged. Samson no longer attacks Kelson, and the two develop a human connection as his humanity begins to resurface.
+The Fingers raid a farm inhabited by survivors, including Tom and his pregnant partner, Cathy. From a distance, Jimmy Ink catches sight of the Bone Temple, and Kelson dancing with Samson. In a barn, Cathy hides as Sir Jimmy orders the Fingers to skin the captured survivors alive as a sacrifice to Old Nick, claiming that Satan is his father.
+Running low on sedatives, Kelson prepares to euthanise Samson, but is overjoyed when Samson says his first word, "moon", suggesting that the Rage Virus may be treatable. Meanwhile, Jimmy Ink, who is growing disillusioned with Sir Jimmy, takes pity on Spike and protects him. Sir Jimmy offers Tom a place in the gang if he can win a death match against a Finger, but Tom is outmatched by his opponent, Jimmima. Cathy breaks her cover to kill Jimmima and Tom sets the barn on fire with a propane tank, killing one of the Fingers before being killed. Sir Jimmy sends Spike to capture Cathy; Spike, traumatised, begs her to take him with her, but Cathy does not trust him, and escapes.
+With the gang's numbers and morale low, Sir Jimmy threatens to kill Spike for his failure to capture Cathy, but Ink suggests they visit Kelson — whom she assumes is Old Nick, having mistaken the iodine for red skin, and Samson as a demon — and let him decide Spike's fate. At the Bone Temple, Sir Jimmy meets Kelson alone and threatens to kill him if Kelson does not pose as Satan and substantiate Sir Jimmy's leadership over the Fingers.
+The next morning, Spike tries to leave Sir Jimmy's camp, but is confronted by Jimmy Fox, who attempts to kill him to avenge Jimmy Shite's death. Ink kills Fox and brings Spike back. Kelson fears that his research on Samson will be cut short and, in a premature attempt to grant him peace, administers him a cocktail of antipsychotics and other drugs, hypothesising that the Rage Virus causes aggression indirectly via psychotic hallucinations. Experiencing some clarity, Samson visits the abandoned train where he hallucinates a childhood memory. When he speaks normally again, a pack of infected attack him; now immune to reinfection, Samson overpowers and kills them all.
+That night, Kelson complies with Sir Jimmy's demands, impersonating Satan in a pyrotechnic-filled performance of Iron Maiden's "The Number of the Beast" while exposing the gang to hallucinogens. Upon recognising Spike, Kelson betrays Sir Jimmy by ordering the Fingers to crucify him. Sir Jimmy fatally stabs Kelson, and Ink is forced to kill the other two Fingers in self-defence. Spike stabs Sir Jimmy, before comforting the dying Kelson. Ink crucifies Sir Jimmy on an inverted cross. Spike and Ink, whose real name is Kellie, leave the Bone Temple. Samson arrives and greets Kelson by name, thanking him as Kelson succumbs to his wounds. Samson carries his body away. After hallucinating Samson as the devil, Sir Jimmy is attacked by an infected.
+Some time later, Spike and Kellie are attempting to escape a group of infected, unaware that they are being observed by Jim, a survivor of the initial outbreak of the Rage Virus, and his teenage daughter, Sam, who break off a history lesson about postwar Europe to go to their aid.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -1015,7 +1074,13 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>The Greek god Hermes welcomes the audience to the show, introducing the story, characters, ensemble, and band ("Road to Hell"). Eurydice and the Fates describe Eurydice’s cynical worldview as well as the harsh weather and famine ("Any Way the Wind Blows"). Orpheus, Hermes' ward, introduces himself to Eurydice and abruptly asks her to marry him ("Come Home with Me"). Eurydice is doubtful, as they both live in poverty.</t>
+          <t>The Greek god Hermes welcomes the audience to the show, introducing the story, characters, ensemble, and band ("Road to Hell"). Eurydice and the Fates describe Eurydice’s cynical worldview as well as the harsh weather and famine ("Any Way the Wind Blows"). Orpheus, Hermes' ward, introduces himself to Eurydice and abruptly asks her to marry him ("Come Home with Me"). Eurydice is doubtful, as they both live in poverty. Orpheus tells her that he is writing a song to make spring come again, and they will no longer have to endure hardship ("Wedding Song").
+Prompted by Hermes, Orpheus tells the story of Hades and Persephone ("Epic I"). Persephone arrives in the world above and celebrates summertime ("Livin' it Up on Top"), while Eurydice begins to fall in love with Orpheus ("All I've Ever Known"). Hades comes early to collect Persephone, who voices her misery at having to return to Hadestown, Hades' underground factory. Despite hearing about the never-ending labor endured by the factory workers, Eurydice is intrigued by the Fates' rich praise of Hadestown, and its promise of protection ("Way Down Hadestown"). The cold weather returns, and Eurydice searches for food and firewood, urging Orpheus to finish his song ("A Gathering Storm"). Orpheus continues working on his song ("Epic II") as Eurydice becomes more desperate as times grow harder.
+After Persephone and Hades argue ("Chant"), Hades leaves Hadestown to find someone who will appreciate its safety and security. He comes across a desperate Eurydice, who has become caught in a snowstorm, and invites her to come to Hadestown ("Hey, Little Songbird"), and the Fates urge Eurydice to join him ("When the Chips Are Down"). With the cold surging and an empty stomach, Eurydice sees no other choice except to follow Hades. She bids goodbye to the preoccupied Orpheus and heads to Hadestown; the Fates chastise the audience for judging her for choosing self-interest over love ("Gone, I'm Gone"). Orpheus realizes Eurydice is missing and resolves to rescue her from Hadestown. Using Hermes' instructions, he travels to Hadestown the long way without the use of the train ("Wait for Me"). As Hades revels in his power and dominion over the denizens of his realm ("Why We Build the Wall"), Eurydice arrives in Hadestown and signs a contract to become a worker in Hadestown.
+Persephone sings to the patrons of a speakeasy that she runs behind Hades's back ("Our Lady of the Underground"). Eurydice begins to recognize the consequences of her choice to go to Hadestown: she will become a forgotten laborer and can never leave unless Hades lets her go ("Way Down Hadestown" (reprise)). Regretting her decision, she begins to forget her life and the world above ("Flowers").
+Orpheus arrives in Hadestown and promises Eurydice that he will take her home ("Come Home with Me" (reprise)). Hades tells him that Eurydice willingly signed the contract and orders the workers to attack Orpheus ("Papers"). The Fates tell him to give up hope ("Nothing Changes"). Orpheus vows to find a way to free Eurydice, rallying the workers and catching Persephone's attention in the process ("If It's True").
+Persephone is inspired by Orpheus's determination and pleads with Hades to let Eurydice go ("How Long?"). While the workers begin to question the freedom they were promised, Hades challenges Orpheus to sing his completed song, threatening to kill him afterwards ("Chant" (reprise)). Orpheus sings his song, reminding Hades of his love for Persephone ("Epic III"). Hades and Persephone reconcile with a dance ("Epic III ('They Danced...')"), after which Orpheus and Eurydice promise to stay together no matter the difficulty ("Promises"). Orpheus asks Hades if they may leave, and Hades tells him that he has not reached a decision. The Fates taunt Hades for his dilemma: If he kills Orpheus and keeps Eurydice captive, they become martyrs, but if he lets them go, he loses control over his workers as they have begun to agitate for their freedom ("Word to the Wise"). Hades lets Orpheus and Eurydice go on one condition: Orpheus must lead them out single file. If he turns around to confirm that Eurydice is following him, she will return to Hadestown and remain there forever ("His Kiss, the Riot").
+Hermes explains the condition to Orpheus and Eurydice, and they begin the long, frightening walk out, as the workers look to them for hope. Persephone and Hades decide to give their own relationship another chance ("Wait for Me" (reprise)). Just as Orpheus reaches the end, he is overcome by doubt and turns around, condemning Eurydice to return to Hadestown ("Doubt Comes In"). Hermes reflects on the somber tale and why it must be told, as the story resets to the beginning, and the company begins to tell it again ("Road to Hell" (reprise)). After the curtain call, the performer playing Persephone leads the cast in honoring Orpheus for his optimism and bravery ("We Raise Our Cups").</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1063,7 +1128,15 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Hamilton narrates Alexander Hamilton's life in two acts, and details among other things his involvement in the American Revolutionary War as an aide-de-camp to George Washington, his marriage to Eliza Schuyler, his career as a lawyer and Secretary of the Treasury, and his interactions with Aaron Burr (the main narrator for most of the musical), which culminates in their duel that ends Hamilton's life. The orphan Alexander Hamilton experiences a difficult early life, but through his wits and the charity of the people of his hometown, he escapes his home—the island of St. Croix—and immigrates to New York City ("Alexander Hamilton").</t>
+          <t>Hamilton narrates Alexander Hamilton's life in two acts, and details among other things his involvement in the American Revolutionary War as an aide-de-camp to George Washington, his marriage to Eliza Schuyler, his career as a lawyer and Secretary of the Treasury, and his interactions with Aaron Burr (the main narrator for most of the musical), which culminates in their duel that ends Hamilton's life.
+The orphan Alexander Hamilton experiences a difficult early life, but through his wits and the charity of the people of his hometown, he escapes his home—the island of St. Croix—and immigrates to New York City ("Alexander Hamilton"). As a student at King's College in 1776, Hamilton meets Aaron Burr, John Laurens, the Marquis de Lafayette, and Hercules Mulligan ("Aaron Burr, Sir"), and impresses them with his rhetorical skills ("My Shot"). The latter three and Hamilton affirm their revolutionary goals to each other, while Burr remains apprehensive ("The Story of Tonight"). Later, the daughters of the wealthy Philip Schuyler—Peggy, Angelica, and Eliza—go into town and share their excitement about the upcoming revolution ("The Schuyler Sisters"), while loyalist bishop Samuel Seabury argues against the revolution ("Farmer Refuted") and King George III insists on his authority ("You'll Be Back"). During the New York and New Jersey campaign, Hamilton accepts a position as George Washington's aide-de-camp despite longing for field command ("Right Hand Man").
+At a ball hosted by Philip Schuyler ("A Winter's Ball"), Eliza falls helplessly in love with Hamilton, who reciprocates her feelings to the point of marriage ("Helpless"), as Angelica suppresses her own feelings for the sake of their happiness ("Satisfied"). After the wedding, Burr and Hamilton congratulate each other's successes ("The Story of Tonight (Reprise)"), and Burr reflects on Hamilton's swift rise compared to his own more cautious career, as well as his affair with Theodosia, the wife of a British officer ("Wait for It").
+As conditions worsen for the Continental Army with the Battle of Monmouth ("Stay Alive"), Hamilton aids Laurens in a duel against disgraced Major General Charles Lee ("Ten Duel Commandments"), for which Washington suspends him from the army ("Meet Me Inside"). Back home, Eliza reveals that she is pregnant with their first child, Philip, and asks Hamilton to slow down to take in the good that has happened in their lives ("That Would Be Enough"). Lafayette convinces Washington to recall Hamilton and grant him field command for the Battle of Yorktown ("Guns and Ships"). Knowing that Hamilton would die a martyr, Washington tells him that he should carefully consider his actions because whatever he does will be remembered for all time ("History Has Its Eyes on You"). At Yorktown, Hamilton works with Lafayette to take down the British and reveals that Mulligan has been working as a spy, helping them trap the British and win the war ("Yorktown (The World Turned Upside Down)").
+Soon after the victory of Yorktown, King George asks the newborn America how it will succeed on its own ("What Comes Next?"). Hamilton's son Philip is born, while Burr has a daughter, Theodosia, and the two new fathers promise their children that they will do anything to protect them ("Dear Theodosia"). Hamilton receives word that Laurens has been killed in a pointless battle with evacuating British troops after the war was already over and responds to his grief by throwing himself into his work ("Tomorrow There'll Be More of Us (The Laurens Interlude)"). Over the next decade, both Hamilton and Burr return to New York and work as lawyers. Through his work and writing, Hamilton rapidly gains influence, participates in the Constitutional Convention, co-authors The Federalist Papers and is selected as Secretary of the Treasury by newly elected President Washington, amidst Eliza begging him to slow down and Angelica moving to London with her new husband ("Non-Stop").
+In 1789, Thomas Jefferson returns to America from being the U.S. ambassador to France, taking up his newfound position as Secretary of State ("What'd I Miss"). Jefferson and James Madison debate against Hamilton's financial proposals at a Cabinet meeting. Washington orders Hamilton to figure out a compromise to push his plan through Congress ("Cabinet Battle #1"). Eliza and her family—along with Angelica, visiting from London—travel upstate during the summer, while Hamilton stays home to work on the compromise ("Take a Break"). Hamilton begins an affair with Maria Reynolds, making him vulnerable to her husband's extortion ("Say No to This"). Hamilton, Jefferson, and Madison finally reach a compromise over a private dinner: they will push through Hamilton's financial plan in exchange for placing the country's permanent capital on the Potomac River. Burr is envious of Hamilton's sway in the government and wishes that he had similar power ("The Room Where It Happens"). Burr switches political parties and defeats Hamilton's father-in-law Philip Schuyler in a race for the Senate, now making Hamilton a rival ("Schuyler Defeated").
+In another Cabinet meeting, Jefferson and Hamilton argue over whether the United States should assist France in its conflict with Britain. President Washington ultimately agrees with Hamilton's argument for remaining neutral ("Cabinet Battle #2"). In the wake of this, Jefferson, Madison, and Burr decide to join forces to find a way to discredit Hamilton ("Washington on Your Side"). Washington retires from the presidency after his second term, and Hamilton assists in writing his farewell address ("One Last Time"). A flabbergasted King George receives word that George Washington has stepped down, and will be replaced by John Adams ("I Know Him"). Adams fires Hamilton, who, in response, publishes an inflammatory critique of the new president ("The Adams Administration").
+Jefferson, Madison, and Burr confront Hamilton about James Reynolds's blackmail years earlier, accusing him of embezzlement ("We Know"). Desperate to salvage his political career by proving that he was merely lustful and not corrupt, Hamilton reminisces over his life and how writing has always saved him ("Hurricane"), before preemptively publicizing his affair in the Reynolds Pamphlet, which wrecks his own reputation ("The Reynolds Pamphlet"). It also ruins his relationship with Eliza, who, in heartbroken retaliation, burns all the letters Hamilton wrote her, trying to erase herself from history ("Burn"). At 19 years old, Hamilton's son Philip attempts to defend his father's honor in a duel with George Eacker ("Blow Us All Away"), but is fatally shot ("Stay Alive (Reprise)"), eventually leading to reconciliation between Alexander and Eliza ("It's Quiet Uptown").
+Hamilton's surprising endorsement of longtime political enemy Jefferson over Burr in the 1800 presidential election ("The Election of 1800") dramatically intensifies the animosity between Hamilton and Burr, who reaches his breaking point and challenges Hamilton to a duel via an exchange of letters ("Your Obedient Servant"). Hamilton writes his last letter in a rush while Eliza tells him to go back to bed ("Best of Wives and Best of Women"). Burr reflects on the events leading up to the duel, while Hamilton reflects on his legacy, before firing his bullet up in the air. Burr fatally shoots Hamilton, and laments that though he survived, he is destined to be remembered by history as the villain who killed Hamilton ("The World Was Wide Enough"). The musical closes with a reflection on historical memory. Jefferson and Madison reflect on Hamilton's legacy, while Eliza tells how she reinserted herself in history and ensured Hamilton's memory by recording the memories of fellow veterans, raising funds for the Washington Monument, speaking out against slavery, and establishing the first private orphanage in New York City ("Who Lives, Who Dies, Who Tells Your Story"). Finally, alone on stage, Eliza turns toward the audience and quietly weeps.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -1111,7 +1184,15 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Mrs. Wormwood gives birth to Matilda, but the new mother is only worried about a ballroom dancing contest she has missed. Similarly shallow, Mr. Wormwood—a used-car salesman and scam artist dismisses the child when he realizes she is a girl ("Miracle"). Five years later, Matilda is an avid reader and lives unhappily with her parents and her older brother Michael. The Wormwoods are oblivious to her genius and frequently mock and verbally abuse her.</t>
+          <t>Mrs. Wormwood gives birth to Matilda, but the new mother is only worried about a ballroom dancing contest she has missed. Similarly shallow, Mr. Wormwood—a used-car salesman and scam artist dismisses the child when he realizes she is a girl ("Miracle"). Five years later, Matilda is an avid reader and lives unhappily with her parents and her older brother Michael. The Wormwoods are oblivious to her genius and frequently mock and verbally abuse her. They prefer to watch TV over reading. Matilda adds some of her mother's peroxide to her father's hair oil, leaving Mr. Wormwood with bright green hair ("Naughty").
+At the library, Matilda spends time with the kind librarian Mrs. Phelps and makes up a story about a world famous acrobat and escapologist who cannot have children. Out of despair, the couple decide to put on a show containing a very dangerous act ("Once Upon a Time"). Matilda has her first day at school ("School Song"). Her teacher Miss Honey instantly sees that Matilda is exceptionally intelligent and decides to request that Matilda be moved to the top class ("Pathetic"). However, the child-hating and tyrannical headmistress Miss Trunchbull dismisses Miss Honey's suggestion. Miss Trunchbull explains that Matilda is better off in Miss Honey's class. Miss Trunchbull doesn't feel that Matilda is ready to be in the top class. ("The Hammer")
+Matilda's father takes out his career frustration on Matilda, so she puts superglue around the rim of his hat. At school, Matilda is told of Miss Trunchbull's cruel punishments, including The Chokey: a tiny cupboard lined with sharp objects in which she locks disobedient children for hours ("The Chokey Chant"). After Matilda meets her best friend Lavender and saves their friend Nigel from Miss Truncbhull when he's accused of putting syrup on her chair, Miss Trunchubll throws their classmate Amanda Thripp over the fence by her hair as punishment for wearing pigtails. Later, Miss Honey meets Mrs. Wormwood and her dance partner Rudolpho. Mrs. Wormwood mocks Matilda's interest in books and intellect ("Loud"). Miss Honey is desperate to help Matilda but feels powerless to do so ("This Little Girl").
+Continuing her story, Matilda explains that the escapologist announces that their act is canceled because the acrobat is pregnant, but her sister refuses to cancel the show and refund tickets, and produces a contract legally binding them to perform the act or go to prison ("The Great Day Arrived"). At school, Miss Trunchbull attempts to accuse Matilda of eating a chocolate cake she had been saving, but quickly learns that the student who ate the cake was Bruce Bogtrotter. As punishment, she forces him to eat an entire chocolate cake as the rest of the students watch him, half of them anticipating that he'll eat the entire cake, while the others are doubtful ("Bruce"). Even though Bruce manages to finish the entire cake, Miss Trunchbull still sends him to The Chokey.
+Mr. Wormwood advises the audience against reading in favour of watching television ("Telly"). Matilda's classmates sing about their hopes for the future ("When I Grow Up"). Matilda tells Mrs. Phelps more of the story of the acrobat and the escapologist. Legally bound by their contract, they perform their act. The acrobat is fatally injured, living just long enough to give birth to a girl. The acrobat asks her husband to take care of their daughter and love her. After giving birth, the acrobat dies from her injuries. The escapologist invites the acrobat's sister to move in and look after his daughter. The girl's aunt is secretly cruel to her niece. The aunt blames the girl for her sister's death ("The Trick Started Well").
+Mr. Wormwood is pleased because he tricked his Russian customers ("I'm So Clever"). Matilda scolds him, so he locks her in her bedroom. Matilda continues the story of the acrobat and escapologist's daughter. The aunt locks her in the cellar, where the father finds her crying. Filled with rage, he goes to confront the aunt but is never seen again. He dies off stage and the aunt becomes the girl's legal guardian ("I'm Here").
+The next day, Miss Trunchbull forces Miss Honey's class to undergo a gruelling physical education lesson ("The Smell of Rebellion"). Miss Trunchbull bullies the children, then verbally abuses Matilda, but Matilda discovers she can move objects with her mind ("Quiet"). Matilda demonstrates her powers to Miss Honey who tells of her own cruel and abusive aunt, who looked after her as a child after her parents died. When Miss Honey first became a teacher, her aunt produced a bill detailing everything Miss Honey consumed as a child, along with other expenses, and forced her to sign a contract binding her to pay it all back. Desperate to escape, Miss Honey found refuge in an old farm shed ("My House"). Matilda recognizes Miss Honey's scarf from the story of the acrobat and the escapologist which she realizes is the true story of Miss Honey's childhood, and that her wicked aunt is Miss Trunchbull.
+Miss Trunchbull schemes to punish Lavender for putting a newt in the jug of water she usually drinks from, but her classmates try to intervene. Matilda uses her powers to write on the blackboard posing as the ghost of Miss Honey's father ("Chalk Writing"). Miss Trunchbull runs away and the children celebrate ("Revolting Children").
+Miss Honey receives her parents house and money, and she becomes the new headmistress. Matilda can no longer use her powers. The Wormwoods try to escape with Michael and Matilda to Spain but the Russian mafia arrive. Sergei is impressed by Matilda's intellect, and he lets them go ("This Little Girl" reprise). Matilda is allowed to live with Miss Honey as the Wormwoods leave for Spain ("When I Grow Up" (reprise)/"Naughty" (reprise)).</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1159,7 +1240,15 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Evan Hansen, a 17-year-old high school senior in Maryland with social anxiety and depression, is assigned by his therapist to write letters to himself detailing what will be good about each day, starting each with "Dear Evan Hansen, today is going to be a good day, and here's why". Evan's overworked mother, Heidi, suggests that Evan, having fallen out of a tree and broken his arm, ask people to sign his cast to make friends. Meanwhile, Cynthia and Larry Murphy struggle to connect with their own 17-year-old son, Connor, a sullen and equally depressed drug abuser who is abusive to his younger sister, Zoe ("Anybody Have a Map?"). At school, Evan meets compulsively-overachieving classmate Alana Beck and his reluctant "family friend" Jared Kleinman, both of whom neglect to sign his cast.</t>
+          <t>Evan Hansen, a 17-year-old high school senior in Maryland with social anxiety and depression, is assigned by his therapist to write letters to himself detailing what will be good about each day, starting each with "Dear Evan Hansen, today is going to be a good day, and here's why". Evan's overworked mother, Heidi, suggests that Evan, having fallen out of a tree and broken his arm, ask people to sign his cast to make friends. Meanwhile, Cynthia and Larry Murphy struggle to connect with their own 17-year-old son, Connor, a sullen and equally depressed drug abuser who is abusive to his younger sister, Zoe ("Anybody Have a Map?").
+At school, Evan meets compulsively-overachieving classmate Alana Beck and his reluctant "family friend" Jared Kleinman, both of whom neglect to sign his cast. Evan runs into Connor, who misinterprets his awkwardness for hostility and pushes him to the ground. Zoe, with whom Evan is infatuated, feels obliged to apologize for her brother's behavior. Evan wonders if his destiny in life is to always be ignored ("Waving Through a Window"). Evan writes the letter to himself in the school library, wondering how he could talk to Zoe and if anyone at school would notice if he disappeared ("Waving Through a Window" [Reprise #1]). Connor bumps into Evan again, this time ironically offering to sign Evan's cast. He finds Evan's letter on the printer and, thinking that Evan intentionally made the letter so Connor would find it, becomes furious and storms out, taking the letter with him. Meanwhile, Alana ponders her own inner anxieties ("Waving Through a Window" [Reprise #2]).
+A few days later, Evan is called to the principal's office, where Connor's parents tell him that their son has died by suicide. They found Evan's letter in Connor's pocket, and mistakenly believe it is a suicide note Connor wrote to Evan. Despite Evan's fumbling attempts to explain the truth, the Murphys believe the two boys had a close friendship and invite Evan to their house for dinner. There, Evan tells them what he thinks they want to hear to avoid discomfort, pretending that he and Connor had secretly been best friends, and recounting a fictional version of the day he broke his arm at an abandoned apple orchard the family had visited years ago ("For Forever"). Evan enlists Jared's help in creating fake, backdated email conversations between him and Connor ("Sincerely, Me").
+After Evan shows the Murphys the fake emails, Cynthia is ecstatic to "learn" that her son had a friend, but Larry is hurt, believing Connor took his family and his privileged life for granted, and Zoe still refuses to mourn Connor because of how he abused her ("Requiem"). However, after reading the "suicide note", Zoe notices that she is mentioned fondly and asks Evan why Connor would say that about her, so he tells her all the reasons he likes her under the guise of Connor saying them ("If I Could Tell Her"). Evan impulsively tries to kiss Zoe, but she pulls away.
+Disgusted by the idea of Connor being forgotten, and motivated by Alana and a vision of Connor, Evan enlists Alana and Jared's help in founding "The Connor Project" to keep Connor's memory alive, which the Murphys eagerly encourage ("Disappear"). While making a speech at a school assembly for Connor, Evan suffers from a panic attack but composes himself, and the speech goes viral online; Zoe, overcome by the impact her brother and Evan have had, kisses him ("You Will Be Found").
+Evan and Alana pitch a fundraising campaign on The Connor Project's website, to raise $50,000 to restore the abandoned apple orchard. Meanwhile, Jared continues to help Evan write fabricated emails, narrowly avoiding a fabricated incest subplot from Jared ("Sincerely Me" [Reprise]). After Heidi learns about Evan's speech about Connor online, she asks him why she never knew about this or the "friendship", and they get into a fight. Evan runs to the Murphys' house, where he bonds with Larry, who offers Evan Connor's old, unused baseball glove ("To Break In a Glove"). While on a date in his house, Evan offhandedly mentions that Heidi is struggling for funds to pay for his college ("Only Us"). Evan becomes preoccupied with Zoe and neglects Heidi, Jared, and The Connor Project. 
+On one of his many visits to the Murphys, Evan finds Zoe invited Heidi for dinner. The Murphys reveal they want to give Connor's college fund to Evan, offending Heidi that Evan would discuss her money troubles with others. At home, Heidi and Evan fight, with Evan telling her he has found family in her absence. Heidi, Alana, and Jared converge in Evan's conscience, compounding his guilt and doubt over his decisions ("Good for You"). Evan debates with the vision of Connor about whether he should tell the truth, where it’s revealed that Evan intentionally fell from the tree in his own suicide attempt ("For Forever" [Reprise]).
+Alana has become suspicious about Evan's "friendship" with Connor, so Evan shows her Connor's "suicide note" to try and prove it. Realizing that the letter is the key to fulfilling the fundraising goal for The Connor Project, Alana posts it online without Evan’s consent. This also goes viral and achieves the goal, but the public begins to blame Connor's wealthy, previously dysfunctional family for his suicide ("You Will Be Found" [Reprise]), making them the targets of harassment. Evan walks in on the Murphys fighting among themselves about the blame and finally admits to them his fabrication; as the Murphys leave in disgust, Evan absorbs his perceived brokenness as inescapable ("Words Fail"). Heidi recognizes the "suicide note" online as one of Evan's therapy assignments and apologizes to him for not seeing how badly he has been hurting. She recalls the day his father moved out and promises that she will always be there for him when he needs her ("So Big/So Small").
+A year later, Evan is still living with his mother, working at a store to earn enough money for college the next semester. Zoe invites him to meet her at the orchard, which has been reopened. He apologizes for the pain he caused and Zoe forgives him, saying the ordeal brought her family closer together. After they part ways, Evan mentally writes himself one last letter reflecting on the impact he has had on his community and questions what is to come next ("Finale").</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1207,7 +1296,16 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>The citizens of Oz are celebrating the death of the Wicked Witch of the West. Glinda the Good Witch appears and reminisces about their past, beginning with the troubled childhood of the Witch (born Elphaba Thropp) after her mother had an affair and her father, the Governor of Munchkinland, disowned her when she was born with green skin ("No One Mourns the Wicked"). Flashing back many years earlier, Elphaba arrives at Shiz University with her younger paraplegic sister Nessarose, where she is ostracized for her green skin and sarcastic personality ("Dear Old Shiz"). The school's headmistress, Madame Morrible, assigns Elphaba to room with the popular Galinda Upland.</t>
+          <t>The citizens of Oz are celebrating the death of the Wicked Witch of the West. Glinda the Good Witch appears and reminisces about their past, beginning with the troubled childhood of the Witch (born Elphaba Thropp) after her mother had an affair and her father, the Governor of Munchkinland, disowned her when she was born with green skin ("No One Mourns the Wicked").
+Flashing back many years earlier, Elphaba arrives at Shiz University with her younger paraplegic sister Nessarose, where she is ostracized for her green skin and sarcastic personality ("Dear Old Shiz"). The school's headmistress, Madame Morrible, assigns Elphaba to room with the popular Galinda Upland. Recognizing Elphaba's magical potential, Morrible decides to privately tutor Elphaba in sorcery ("The Wizard and I"), making Galinda intensely jealous. The two girls soon come to loathe each other ("What Is This Feeling?"). Meanwhile, Dr. Dillamond, the only animal professor at Shiz, informs Elphaba of a conspiracy to stop all animals from speaking ("Something Bad").
+A roguish prince, Fiyero, begins attending Shiz and arranges a party for his fellow students. Galinda becomes immediately enamored with him, and convinces her admirer, the Munchkin Boq, to take Nessarose to the party instead so that she can go with Fiyero. At Nessarose's urging, Elphaba asks Morrible to begin teaching Galinda sorcery. When Elphaba is mocked at the party for wearing an ugly hat Galinda gave her as a practical joke, Galinda has a change of heart and decides to dance with Elphaba ("Dancing Through Life"). In their room, the girls finally bond and Galinda gives Elphaba a makeover ("Popular"). The next day, Dillamond tells the class he has been dismissed. His human replacement showcases a cage, a new invention in Oz designed to stop animals from speaking. Elphaba, furious, frees the lion cub imprisoned within it and escapes with Fiyero. They share a private moment, but Elphaba laments that Fiyero has chosen Galinda ("I'm Not That Girl").
+Morrible tells Elphaba that the Wizard of Oz wants to meet her, and she goes with Galinda, who changes her name to Glinda in honor of Dillamond (who mispronounced her name as such), to the Emerald City ("One Short Day"). The two meet the Wizard and are surprised to discover his mortal nature ("A Sentimental Man"). Morrible appears and announces she is the Wizard's new press secretary. After being tricked into enchanting the Wizard's monkey servants to painfully sprout wings, Elphaba deduces that the Wizard is behind the suppression of animals and is a fraud who uses parlor tricks and lies to stay in power. Elphaba flees his chambers, declaring against Glinda's wishes that she must do what is right. Though empathetic, Glinda refuses to leave with Elphaba, and the two friends bid farewell before Elphaba enchants a broom to fly away from the Emerald City, vowing to fight the Wizard with all of her power ("Defying Gravity").
+Years later, Elphaba has become known as the Wicked Witch of the West for her opposition to the Wizard's regime, while Glinda has been positioned by Madame Morrible as the Wizard's spokesperson. Fiyero, now Captain of the Wizard's Guard and unwitting fiancé to Glinda, hopes to find Elphaba ("Thank Goodness").
+Elphaba visits Nessarose, who is now the governor of Munchkinland following their father's death and has removed the Munchkins' few rights to prevent Boq from leaving her. Feeling guilty, Elphaba enchants Nessa's silver shoes to allow her to walk, but Boq takes this as proof that Nessarose no longer needs him and attempts to leave her for Glinda. An infuriated Nessarose attempts to cast a love spell on him, but pronounces the incantation wrong and shrinks his heart instead. Elphaba tries to save him, but can only transform him into a tin man who does not need a heart to live ("The Wicked Witch of the East"). Boq flees as Nessarose blames Elphaba.
+Elphaba returns to the Emerald City to free the Wizard's monkey servants, but the Wizard discovers her. He once again tries to convince Elphaba to work with him, explaining he is an ordinary man who became revered by the citizens of Oz ("Wonderful"), and voluntarily frees the monkeys. Elphaba is won over until she discovers a caged Dillamond, who has lost the ability to speak, and vows to continue her fight against the Wizard. Fiyero helps Elphaba escape and decides to leave with her. Glinda is heartbroken and spitefully suggests spreading a rumor that Nessarose is in danger to lure Elphaba out of hiding, before privately lamenting that Fiyero always loved Elphaba ("I'm Not That Girl (Reprise)"). Unbeknownst to Glinda, Morrible and the Wizard decide a mere rumor would not fool Elphaba, and Morrible proposes "a change in the weather."
+Hidden in the forest, Elphaba and Fiyero proclaim their love to each other ("As Long as You're Mine"), but their moment is shattered when Elphaba senses that Nessarose is in danger. She rushes back to Munchkinland to find that a house has fallen from a tornado and crushed her sister to death. Elphaba is distraught and furious that Glinda has given Nessarose's enchanted shoes to the house's occupant, Dorothy Gale, and the two get into a physical fight that the Wizard's guards eventually break up. Fiyero arrives and allows Elphaba to escape, but the guards arrest and torture him for her whereabouts. At Kiamo Ko castle, Elphaba casts a spell to try to save Fiyero; presuming him dead, she laments that she will never be seen as good and finally embraces her reputation as the Wicked Witch of the West ("No Good Deed").
+As the Citizens of Oz declare war on Elphaba ("March of the Witch Hunters"), Glinda realizes that Morrible summoned the tornado that killed Nessarose and is horrified, but Morrible reminds her that she has been complicit in all of Morrible and the Wizard's plans to further her own goal of becoming a powerful figure in Oz. Meanwhile, Elphaba, crazed with grief, has captured Dorothy to try to obtain Nessarose's shoes. Glinda arrives to warn Elphaba of her danger. Elphaba accepts that she must surrender, and the two friends embrace for the last time before sharing a tearful goodbye ("For Good"). Glinda watches from the shadows as Dorothy throws a bucket of water on Elphaba, apparently melting her and leaving only her hat and a bottle of Green Elixir that had belonged to her mother.
+Glinda confronts the Wizard with the elixir, which he recognizes as his own; he was the man Elphaba's mother had an affair with and thus her biological father. The Wizard leaves Oz at Glinda's orders, leaving her in charge, and she arrests Morrible for her role in Nessarose's death. Meanwhile, Fiyero (now a Scarecrow as the result of Elphaba's spell) arrives at Kiamo Ko, where Elphaba emerges from a trap door, having faked her death. Elphaba and Fiyero depart Oz together, as Glinda informs everyone that the Wicked Witch is dead before reluctantly joining Oz in celebrating ("Finale").</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -1255,7 +1353,20 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>As the sun rises, Rafiki the mandrill calls the animals to Pride Rock. She greets King Mufasa and Queen Sarabi before presenting their cub to the gathered animals ("Circle of Life"). Elsewhere, Mufasa's brother, Scar, laments his lost chance at becoming King. Back at her baobab tree, Rafiki paints an image of the cub and asks the spirits to conjure the new prince's name: Simba.</t>
+          <t>As the sun rises, Rafiki the mandrill calls the animals to Pride Rock. She greets King Mufasa and Queen Sarabi before presenting their cub to the gathered animals ("Circle of Life"). Elsewhere, Mufasa's brother, Scar, laments his lost chance at becoming King. Back at her baobab tree, Rafiki paints an image of the cub and asks the spirits to conjure the new prince's name: Simba.
+Time passes and Simba grows into a lively young cub ("Grasslands Chant"). Mufasa shows Simba the Pride Lands from the top of Pride Rock and explains that everything exists in a delicate balance known as the Circle of Life. Mufasa warns Simba not to stray beyond the boundaries of the Pride Lands, pointing out a shadowy area in the distance. Zazu, a hornbill who acts as Mufasa's advisor, arrives and delivers his daily report on the state of affairs in the King's domain ("The Morning Report", now cut from the Broadway production).
+Simba goes to see his Uncle Scar. The scheming lion piques the cub's curiosity by mentioning the elephant graveyard, where Simba is forbidden to go. Meanwhile, the lionesses go hunting ("The Lioness Hunt"). Simba arrives and asks his best friend, a female cub named Nala, to come with him to the elephant graveyard. He lies to the lionesses about where they are going, and Sarafina (Nala's mother) and Sarabi allow the cubs to go, escorted by Zazu. Simba and Nala formulate a plan and manage to lose Zazu, while Simba brags about his future position ("I Just Can't Wait to Be King").
+The cubs go to the graveyard and begin to explore. Zazu catches up, but they are confronted by three hyenas: Shenzi, Banzai and Ed. The hyenas intend to eat the trespassers and they gloat about their find ("Chow Down"). Mufasa rescues the cubs and frightens off the hyenas.
+Mufasa is disappointed and angry at Simba's reckless disobedience, and explains the difference between bravery and bravado. Mufasa tells Simba about the great kings of the past and how they watch over everything from the stars ("They Live in You"). Mufasa says that he will always be there for his son. Later he discusses Simba's behavior with Zazu, who reminds Mufasa that he had the same tendency to get into trouble at Simba's age.
+Back at the elephant graveyard, Scar tells the hyenas of his plan to kill Mufasa and Simba so that he can become king. He raises an army of hyenas, promising that they will never go hungry again if they support him ("Be Prepared"). Scar takes Simba to a gorge and tells him to wait there. On Scar's signal, the hyenas start a wildebeest stampede into the gorge ("The Stampede"). Scar tells Mufasa that Simba is trapped in the gorge. Mufasa leaps into the stampede and manages to save his son, but as he tries to escape, Scar throws him off the cliff back into the stampede, killing him. Scar convinces Simba that his father's death was his fault and tells him to run away, but as he leaves, Scar orders the hyenas to kill him. Simba escapes but the hyenas tell Scar that he is dead. Rafiki and the lionesses mourn the deaths ("Rafiki Mourns"). Scar claims the throne and allows the hyenas into the Pride Lands ("Be Prepared (Reprise)"). Rafiki returns to her tree and smears the drawing of Simba, while Sarabi and Nala quietly grieve.
+Out in the desert, Simba collapses from heat exhaustion. Vultures begin to circle, but are scared away by Timon the meerkat and Pumbaa the warthog. Simba feels responsible for Mufasa's death, but the duo take the cub to their jungle home and show him their carefree way of life and bug diet ("Hakuna Matata"). Simba grows to adulthood in the jungle.
+The chorus, dressed in colorful clothes with ornate bird puppets and kites, begin the second act ("One by One").  As the song ends, however, the beautiful birds are replaced by vultures and gazelle skeletons. Under Scar's rule, the Circle of Life is out of balance and a drought has hit the Pride Lands. Zazu, now a prisoner of Scar, listens to the king's woes. The hyenas are complaining about the lack of food, but Scar is only concerned with himself and why he is not loved. He is haunted by visions of Mufasa and rapidly switches between delusional confidence and paranoid despair ("The Madness of King Scar"). Nala arrives to confront Scar about the famine and Scar decides she will be his queen and give him cubs. Nala fiercely rebukes him and resolves to leave the Pride Lands to find help. Rafiki and the lionesses bless her for her journey ("Shadowland").
+Back in the jungle, Timon and Pumbaa want to sleep, but the restless Simba is unable to settle. Annoyed, Simba leaves them, but Timon and Pumbaa lose their courage and follow him. Simba leaps across a fast-moving river and challenges Timon to do the same. Timon falls in and is swept downstream. He grabs a branch over a waterfall and calls for Simba's help, but Simba is paralyzed by a flashback of Mufasa's death. Timon falls from the branch and Simba snaps out of the flashback, rescuing his friend. Simba is ashamed that Timon nearly died because of his recklessness.
+The three friends settle to sleep and discuss the stars. Simba recalls Mufasa's words, but his friends laugh at the notion of dead kings watching them. Simba leaves, expressing his loneliness and bitterly recalling Mufasa's promise to be there for him ("Endless Night"). Rafiki hears the song on the wind, joyfully realizes that Simba is alive, and draws a mane onto her painting of Simba.
+In the jungle, Pumbaa is hunted and chased by a lioness. Simba confronts her and saves his friend, but recognizes the lioness as Nala. She is amazed to find Simba alive, knowing that he is the rightful king. Timon and Pumbaa are confused, but Simba asks them to leave him and Nala alone. Timon realizes what is happening and laments the end of Simba's Hakuna Matata lifestyle ("Can You Feel the Love Tonight"). Nala tells Simba about the devastated Pride Lands, but Simba still feels responsible for Mufasa's death and refuses to return home.
+On his own, Simba meets Rafiki, who explains that his father lives on ("He Lives in You"). Mufasa's spirit appears in the sky and tells Simba he is the one true king and must take his place in the Circle of Life. Reawakened, Simba finds his courage and heads for home. Meanwhile, Nala wakes Timon and Pumbaa to ask where Simba is, and Rafiki appears to tell them all the news. The three of them catch up with him in the Pride Lands, where he witnesses the ruin of his home. Timon and Pumbaa distract some hyenas by doing the Charleston, allowing Simba and Nala to reach Pride Rock.
+Scar calls for Sarabi and demands to know why the lionesses are not hunting. Sarabi stands up to him about the lack of anything to hunt, angrily comparing him to Mufasa, and Scar strikes his sister-in-law, saying he's ten times the king Mufasa was. Enraged, Simba reveals himself. Scar forces a confession of murder from Simba and corners him. Believing that he has won, Scar taunts Simba by admitting that he killed Mufasa. Furious, Simba recovers and forces Scar to reveal the truth to the lionesses ("Simba Confronts Scar"). Simba's friends fight the hyenas while Simba battles Scar to the top of Pride Rock. Scar begs for his life, blaming the hyenas for everything. Simba lets him leave out of mercy, but Scar attacks again. Simba blocks the attack and Scar falls from the cliff. The hyenas, who heard Scar's betrayal and are still starving, tear him to shreds.
+With the battle won, Simba's friends come forward and acknowledge Simba as the rightful king. Simba ascends Pride Rock and roars out across the kingdom ("King of Pride Rock"). The Pride Lands recover and the animals gather in celebration as Rafiki presents Simba and Nala's newborn cub, continuing the Circle of Life ("Circle of Life (Reprise)").</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1303,7 +1414,17 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>At a Missionary Training Center of the Church of Jesus Christ of Latter-day Saints, devout missionary-to-be Elder Kevin Price leads his classmates in a demonstration of the door-to-door method to convert people to the Church of Jesus Christ of Latter-day Saints ("Hello!"). Price believes if he prays enough, he will be sent to Orlando, Florida, for his two-year mission. However, he learns he will instead be sent to Uganda and paired with Elder Arnold Cunningham, an insecure, pop culture–obsessed compulsive liar ("Two by Two"). Price is sure he is destined to do something incredible, while Cunningham is just happy to follow ("You and Me (But Mostly Me)").</t>
+          <t>At a Missionary Training Center of the Church of Jesus Christ of Latter-day Saints, devout missionary-to-be Elder Kevin Price leads his classmates in a demonstration of the door-to-door method to convert people to the Church of Jesus Christ of Latter-day Saints ("Hello!"). Price believes if he prays enough, he will be sent to Orlando, Florida, for his two-year mission. However, he learns he will instead be sent to Uganda and paired with Elder Arnold Cunningham, an insecure, pop culture–obsessed compulsive liar ("Two by Two"). Price is sure he is destined to do something incredible, while Cunningham is just happy to follow ("You and Me (But Mostly Me)").
+Upon arrival in northern Uganda, the two are robbed by soldiers of a local warlord, General Butt Fucking Naked. The missionaries are welcomed to the village by Mafala Hatimbi. A group of villagers share their daily reality of living in appalling conditions while being ruled by the General. To help them feel better in times of trouble, the villagers repeat a phrase that translates as "Fuck you, God!" ("Hasa Diga Eebowai").
+Price and Cunningham are led to their living quarters by Nabulungi, Mafala's daughter. They meet their fellow missionaries stationed in the area, who have been unable to convert anyone to the Church. Elder McKinley, the district leader, teaches Price and Cunningham to suppress upsetting ideas ("Turn It Off"). By the time they retire for the night, Price is riddled with anxiety, but Cunningham reassures him that he will succeed and that, as his companion, Cunningham will be by his side no matter what ("I Am Here for You").
+Price is confident he can succeed where the other elders have failed, teaching the villagers about Joseph Smith through a song that begins as a tribute to Smith but eventually descends into a tribute by Price to himself ("All-American Prophet"). The General arrives and announces his demand for the genital mutilation of all female villagers. After a villager protests, the General murders him. Taking every last measure to protect her, Mafala commands Nabulungi to stay in their house with all the doors locked and windows closed. She protests, insisting that the women of the village will not have to stay in hiding if they listen to the missionaries, as they hold the secrets to liberation, protection, and eternal happiness. Though her protests to go out and talk to them fail, she calms down after remembering how she was moved by Price's promise of an earthly paradise. She yearns to live in that new land, Salt Lake City, with all of her fellow villagers ("Sal Tlay Ka Siti").
+The mission president has requested a progress report on their mission. Shocked by the execution and the reality of Africa, Price decides to abandon his mission and requests a transfer to Orlando. Meanwhile, ever-loyal Cunningham assures Price that he will follow him anywhere. However, Price unceremoniously dumps him as mission companion ("I Am Here for You [Reprise]"). Cunningham is crushed and alone, but Nabulungi comes to him, wanting to learn more about the Book of Mormon and having convinced the villagers to listen to him. Cunningham finds the courage to take control of the situation ("Man Up").
+Cunningham attempts to teach the Book of Mormon to the villagers, but when they become frustrated and begin leaving, Cunningham quickly develops stories, combining what he knows of LDS Church doctrine with pieces of science fiction and fantasy. Cunningham's conscience (personified by his father, Joseph Smith, Hobbits, Lt. Uhura, Darth Vader, and Yoda) admonishes him, but he rationalizes that if it helps people, it surely cannot be wrong ("Making Things Up Again"). Meanwhile, Price joyfully arrives in Orlando, but then realizes that he is dreaming his childhood nightmares of Hell and sees Jesus, Satan, Genghis Khan, Jeffrey Epstein (it had previously been Jeffrey Dahmer prior to 2026), Adolf Hitler, and Johnnie Cochran, who all call him out on abandoning Cunningham ("Spooky Mormon Hell Dream"). Price awakens and decides to re-commit to his mission.
+Cunningham announces that several Ugandans are interested in the Church, but McKinley explains that unless the General is dealt with, no one will convert. Price, seeing this as his chance to prove his worth, sets off on the "mission he was born to do." After reaffirming his faith, he confronts the General, determined to convert him ("I Believe"). The General is unimpressed and drags Price away.
+Cunningham concludes his preaching, and the villagers are baptized, with Nabulungi and Cunningham sharing a tender moment as they do ("Baptize Me"). The missionaries feel oneness with the people of Uganda and celebrate ("I Am Africa"). Meanwhile, Price is seen in the village doctor's office, having the Book of Mormon removed from his rectum. The General hears of the villagers' conversion and resolves to kill them all.
+Having lost his faith, Price drowns his sorrows in coffee. Cunningham finds Price and tells him they need to at least act like mission companions, as the mission president is coming to visit the Ugandan mission. Price reflects on all the broken promises the Church, his parents, his friends, and life in general made to him ("Orlando").
+Nabulungi and the villagers perform a pageant for the mission president to "honor [him] with the story of Joseph Smith, the American Moses", which reflects the distortions put forth by Cunningham, such as having sex with a frog to cure their AIDS ("Joseph Smith American Moses"). The mission president is appalled, orders all the missionaries to go home, and tells Nabulungi that she and her fellow villagers are not members. Nabulungi, heartbroken at the thought that she will never reach paradise, curses God for forsaking her ("Hasa Diga Eebowai [Reprise]"). Price has an epiphany and realizes Cunningham was right all along: though scriptures are important, what is more important is getting the message across ("You and Me (But Mostly Me) [Reprise]").
+The General arrives, and Nabulungi is ready to submit to him, telling the villagers that Cunningham's stories are untrue. She also explains that they will never see him again, but she protects his reputation in their eyes by saying that a lion ate him. To Nabulungi's shock, they respond that they have always known that Cunningham's stories were metaphors rather than literal truth. Price and Cunningham arrive, and, believing Cunningham to be resurrected from the dead, the General flees. Price rallies the members of the Church and the Ugandans to work together to make this their paradise. Later, the newly minted Ugandan elders (including the General) visit door-to-door to evangelize with "The Book of Arnold" ("Tomorrow Is a Latter Day"/"Hello! [Reprise]").</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1351,7 +1472,11 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>On the morning of September 11, 2001, the townspeople of Gander describe life in Newfoundland and how they learn of the September 11 attacks on the radio ("Welcome to the Rock"). Claude, the mayor of Gander, is informed of the attacks by Janice, a new reporter in town, while at a local Tim Hortons. The town receives the news that the US airspace has been closed, causing US-bound flights to be diverted across Canada, including 38 to Gander International Airport ("38 Planes"). This nearly doubles the population of Gander, and the townspeople make preparations to care for the 7,000 stranded passengers.</t>
+          <t>On the morning of September 11, 2001, the townspeople of Gander describe life in Newfoundland and how they learn of the September 11 attacks on the radio ("Welcome to the Rock"). Claude, the mayor of Gander, is informed of the attacks by Janice, a new reporter in town, while at a local Tim Hortons. The town receives the news that the US airspace has been closed, causing US-bound flights to be diverted across Canada, including 38 to Gander International Airport ("38 Planes"). This nearly doubles the population of Gander, and the townspeople make preparations to care for the 7,000 stranded passengers. Beulah and Annette, two schoolteachers, prepare the local school to take in passengers, while Janice asks for the community to provide resources ("Blankets and Bedding").
+For hours, the plane passengers are forbidden from leaving the planes, and are without information about the attacks. They express frustration and fear at being stranded. A Gander SPCA worker, Bonnie, goes into the plane holds to search for animals on the planes, and Claude reaches an agreement with Garth, a union leader, to pause the bus drivers' strike and transport passengers ("28 Hours/Wherever We Are"). The passengers are eventually transported to Gander and surrounding towns for shelter ("Darkness and Trees"). A Muslim passenger, Ali, is temporarily detained. The local bus drivers take passengers to the towns and explain the culture of Newfoundland while navigating language barriers with international passengers ("On the Bus"/"Darkness and Trees (reprise)"). The passengers learn why they were grounded and watch replays of the attacks on television ("Lead Us Out of the Night"). They attempt to contact their families ("Phoning Home") and experience disorientation and stress at their situation ("Costume Party").
+The town tries to manage food, sanitation, and other necessities for the guests. Some of the passengers try to get home, but are informed by Oz, the constable of Gander, that travel to the US takes several days. Nick, a British passenger, and Diane, a Texan, go for a walk with a gay couple from Los Angeles, both named Kevin. Bonnie and her husband Doug discover two rare bonobo chimpanzees in the hold of a plane. An American, Bob, is asked to take grills from backyards to set up for a community cookout; he fears he will be shot for stealing, but he finds everyone is friendly and willing to help. Hannah, the mother of a New York firefighter, bonds with Beulah and worries about her son ("I Am Here"). Many of the passengers of various religious beliefs go to a local Catholic church or other spaces around town to pray ("Prayer"). Ethnic and national tensions erupt among the passengers and townsfolk ("On the Edge"). To alleviate this, the passengers are invited to a local bar and some are initiated as honorary Newfoundlanders ("Heave Away"/"Screech In"). One pilot who has been diverted, Beverley, reflects on her experience as the first female captain for American Airlines ("Me and the Sky").
+The planes prepare to leave, and Ali is subjected to a strip search prior to leaving on suspicion he may be a terrorist. When flights are delayed, Nick and Diane go for a walk around the town and realize they will miss each other when they leave Gander ("The Dover Fault"/"Stop the World"). When the planes are cleared for takeoff, the passengers express happiness at returning to the US, and set up a donation fund for the people of Gander ("38 Planes" (reprise)"/"Somewhere in the Middle of Nowhere"). After the events of the last five days, both the townspeople and passengers experience loneliness and fear about the state of the world; the two Kevins' relationship has fallen apart due to the stress of the crisis, and Hannah is devastated to learn her son has died ("Something's Missing"). 
+Ten years after the attacks, the townspeople and the passengers reunite in Gander (including Diane and Nick, who have since married) and celebrate the relationships formed while the passengers were stranded ("Ten Years Later"/"Finale").</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1455,7 +1580,25 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Five versions of the libretto of Anything Goes exist: the original 1934 libretto, the 1962 off-Broadway revival libretto, the 1987 revival libretto, the 2011 revival libretto, and the 2022 revised libretto. The story has been revised, though all involve similar romantic complications aboard the SS American and feature the same major characters. The score has been altered, with some songs cut and others reassigned to different scenes and characters, and augmented with various Porter songs from other shows. Billy Crocker, a young Wall Street broker, has fallen in love with a beautiful girl he met at a party and spent the evening with in a taxi.</t>
+          <t>Five versions of the libretto of Anything Goes exist: the original 1934 libretto, the 1962 off-Broadway revival libretto, the 1987 revival libretto, the 2011 revival libretto, and the 2022 revised libretto. The story has been revised, though all involve similar romantic complications aboard the SS American and feature the same major characters. The score has been altered, with some songs cut and others reassigned to different scenes and characters, and augmented with various Porter songs from other shows.
+Billy Crocker, a young Wall Street broker, has fallen in love with a beautiful girl he met at a party and spent the evening with in a taxi. His boss, Elisha J. Whitney, is preparing to make a business deal and is going to travel to London aboard the SS American. Evangelist-turned-nightclub singer Reno Sweeney will be traveling aboard the same ship. Billy sees Reno as a friend, but she obviously has feelings for him ("I Get a Kick Out of You"). Billy goes to the dock to say farewell to his boss and Reno ("Bon Voyage"), and glimpses the mysterious girl again. He learns that she is the heiress Hope Harcourt and, escorted by her mother Mrs. Harcourt, is on her way to England with her fiancé Lord Evelyn Oakleigh, a handsome but stuffy and hapless British nobleman. Billy stows away on the ship with a plan of winning Hope's heart. "Moonface" Martin, a second-rate gangster labeled "Public Enemy 13", and his girlfriend, Bonnie, have disguised themselves as a minister and a missionary and, innocently aided by Billy, board the ship under their assumed identities, stranding the ship's real chaplain back at the port. Moonface and Bonnie mistakenly leave behind their leader, "Snake Eyes" Johnson, Public Enemy 1.
+To thank him, Bonnie and Moonface let Billy have Snake Eyes Johnson's passport and ticket without telling him to whom they belong. Billy cons Evelyn into leaving him alone with Hope, by convincing him he is very ill. When he goes to get some air, Billy and Hope meet again, and it turns out she has been unable to stop thinking about him as well ("All Through the Night"). Though Hope prefers Billy, she insists she must marry Evelyn. Unbeknownst to Billy, her family's company is in financial trouble and a marriage to Evelyn would promote a merger and save it. The ship's crew gets a cable from New York saying that Public Enemy 1 is on board. Moonface admits his true identity to Billy and he and Bonnie conspire to disguise Billy as a crew member since he is now presumed to be Snake Eyes Johnson.
+A quartet of lovelorn sailors comfort themselves with the thought of romance when they reach shore ("There'll Always Be a Lady Fair"). On deck, Bonnie lures the sailors to her ("Where Are the Men?"), then steals the clothes of one of the men for Billy.
+Hope discusses her impending marriage with Evelyn and discovers that he is not particularly pleased with the engagement either. Billy asks Reno to help separate Evelyn and Hope, and she agrees. Billy and Reno reaffirm their friendship ("It's Friendship"). Reno tries to charm Evelyn; she succeeds and he invites her for a drink in his cabin. She and Moon plot that Moon should burst into the cabin and discover Reno half-naked in Evelyn's arms, providing sufficient reason for breaking off the engagement. However, when Moon breaks into the room, machine gun in tow, he instead sees Reno fully dressed and Evelyn nearly undressed. Moon tries to invent some indecent explanation for the situation, but Evelyn insists that he would be quite pleased by any rumor depicting him as a passionate lover, especially if Hope heard it. Moon admits that the plot has failed.
+The crew discover that Billy is not a sailor, and Moon and Reno create a new disguise for him from a stolen pair of trousers, a jacket taken from a drunken passenger, and hair cut from Mrs. Harcourt's Pomeranian and made into a beard. Reno tells Billy that Evelyn has kissed her, and she is sure she will be Lady Oakleigh soon, since love moves so quickly these days ("Anything Goes"). Mrs. Harcourt, recognizing her dog's hair, angrily pulls off Billy's beard and the crew and passengers realize he must be the wanted man. As Snake Eyes Johnson, Billy is an instant celebrity.
+Billy is honored by both crew and passengers as "Public Enemy Number One". He tells the Captain that Moon (who is still disguised as a minister) is helping him reform from his wicked ways. Moon is asked to lead a revival in the ship's lounge. The passengers confess their sins to the "Reverend", and Lord Evelyn admits to a one-night stand with a young Chinese woman, Plum Blossom. Hope is not impressed with Billy's charade, and to please her, he confesses to everyone that he is not really Snake Eyes Johnson. Moon attempts to compensate by revealing that he is not a minister; he is Public Enemy Number Thirteen. The captain sends them both to the brig. Reno restores the mood of the Revival ("Blow, Gabriel Blow").
+Moon tries to cheer Billy up ("Be Like the Bluebird"). Billy doubts he will ever see Hope again; he and Moon cannot leave their cell until they return to America. Their card-playing Chinese cellmates Ching and Ling, imprisoned for conning all the third class passengers out of their money, will be put ashore in England. Moon and Billy challenge them to a game of strip poker, win their clothes, and disguise themselves again.
+Billy, Moon, and Reno show up at the Oakleigh estate in Chinese garb. Billy and Moon tell Oakleigh's uncle that they are the parents of "Plum Blossom" and threaten to publicize Evelyn's indiscretion if he does not marry her. Oakleigh offers to buy them off and Moon gleefully accepts the cash, much to Billy and Reno's chagrin.
+Billy and Reno find Hope and Evelyn, who are both unhappy with the prospect of their matrimony. Hope declares that she desperately wants to marry Billy ("The Gypsy in Me"). Billy spots Whitney and finally learns that Evelyn and Hope's planned marriage is really an awkward business merger. Billy realises that Oakleigh is manipulating them all; Hope's company is really worth millions and Billy informs Whitney of that fact. Whitney offers to buy the firm from Hope at an exorbitant price, and she accepts. The marriage is called off since a merger is now impossible. Billy and Hope get married, as do Reno and Evelyn. A cable from the U.S. government fixes Billy's passport problems and declares Moon "harmless". Moon indignantly pockets Oakleigh's check and refuses to return it.
+Young Wall Street broker Billy Crocker helps his boss Elisha J. Whitney prepare for his trip to London. Eli tells Billy the next morning he is to make a huge sale of a sinking asset. Billy then runs into his friend; evangelist turned night club singer Reno Sweeney who is leaving on the same ship to London. Reno tries to convince Billy to join her, but he refuses and she laments her unrequited love for him ("I Get A Kick Out Of You"). Billy then reveals to Reno he has fallen in love with someone else and she berates him, believing he led her on before sadly reaffirming her feelings for him after he leaves ("I Get A Kick Out Of You - Reprise").
+The next morning the crew of the SS American prepare to set sail ("There's No Cure Like Travel") as Reno and the other passengers board. Among them is debutante Hope Harcourt, the subject of Billy's infatuation. She is joined by her wealthy English fiancé Lord Evelyn Oakleigh and her mother Evangeline, who has set her daughter up to be married in order to solve their family's recent financial struggles. Billy comes aboard to give Eli his passport and spots Hope. Upon hearing that she is to be wed, he stays on the ship in order to pursue her. Also sneaking on to the American is Public Enemy No. 13 Moonface Martin, who is disguised as a priest. He is joined by Erma, the promiscuous girlfriend of Public Enemy #1 Snake Eyes Johnson, who is nowhere to be found. Billy inadvertently helps Moonface evade the FBI. Moonface returns the favor by giving Billy Snake Eyes' ticket as the ship leaves the dock ("Bon Voyage").
+Later that night, Billy bumps into an apologetic Reno who encourages him to go after his real love. When Billy starts to express insecurities about being with Hope, Reno builds up his confidence while playfully putting herself down, and he returns the favor ("You're The Top"). Billy then scares off a seasick Evelyn so he can court Hope away from him ("So Easy To Love"). Though she returns Billy's feeling, Hope insists on maintaining her duty and marrying Evelyn. Once alone though, she repeats his romantic words ("So Easy To Love - Reprise").
+Eli drunkenly sings about his excitement for the trip, reminisces on his days in Yale, and unsuccessfully invites Hope's mother, Evangeline, to spend the night with him ("The Crew Song"). In the next room over, Moonface and Erma are visited by Billy, who hides when the ship's captain comes in and reveals that Billy is believed to be Snake Eyes Johnson. The next morning a quartet of sailors sing about the joy of seeing women as they come ashore ("There'll Always Be a Lady Fair") while Erma steals another seaman's clothes to disguise Billy from the crew and his boss. Reno then encounters her old friend Moonface, shortly after which Evelyn approaches her and reveals himself to be a huge fan. Evelyn invites Reno for tea in his room, which Moonface convinces her to accept so she can seduce Evelyn, which they'll use to blackmail him and break up his engagement. Reno agrees to his plan and they sing about what great friends they are, only to descend into bickering ("Friendship").
+The attempted extortion proves to be a failure, with Reno and Evelyn instead finding themselves utterly charmed by each other. Billy and Moonface then try to frame Evelyn as a madman to Evangeline only for Hope to step in and expose Billy's identity. The crew pursues him while Reno reprimands Hope for ignoring her own happiness and chasing away the man she loves. Hope breaks into tears before Billy returns to serenade her, with her now reciprocating ("It's Delovely"). However, the next morning Hope struggles to tell her mother of her real love and shortly afterwards Billy is apprehended by the crew. The captain then releases Billy to satisfy the celebrity-crazed passengers, and he basks in the fame of being a gangster whilst Moonface blows his cover to do the same. An upset Hope walks away whilst an onlooking Reno leads the ship in a tap dance and remarks that nowadays, "Anything Goes".
+The whole ship has gathered to honor Billy as "Public Enemy No. 1". After unsuccessfully trying to get him and Hope back together, Reno begins her performance for that night. She starts out with a sermon asking passengers to confess their sins. In his confession, Evelyn tells everyone of the time he had casual sex with a Chinese woman named Plum Blossom. Reno then performs a lively gospel number with everyone else joining in ("Blow, Gabriel, Blow") at which point she declares "they've seen the light". The passengers then convince Billy to make a confession, and he reveals that he is not Snake Eyes Johnson and apologizes to Hope. Moonface tries and fails to defend him, and both are thrown in the brig. Reacting to this development, Evangeline moves the wedding up to the next morning on the ship and a heartbroken Hope realizes her chance at true love is over ("Goodbye  Little Dream, Goodbye").
+In the brig, Moonface attempts to cheer up a depressed Billy by telling him to "Be Like The Bluebird". Erma visits them to deliver a letter from Hope where she confesses her feelings for Billy, at which point they both — on separate parts of the ship — express their love ("All Through The Night"). Reno then meets Evelyn on the deck where he admits that he doesn't love Hope and hints that he has fallen for her instead. Despite this, his sense of honor and family code causes him to keep the engagement. Reno then notes that his one night stand in China contradicts this. At her prodding, Evelyn reveals his Romani ancestry and the wild side he'd previously tried to keep hidden. He shows his true feelings for her, she requites them, and they have a passionate tango dance ("Gypsy In Me").
+Two Chinese passengers are thrown into the brig with Billy and Moonface for gambling. Reno then comes to tell her friends that she and Evelyn have fallen in love with each other. Knowing that the Chinese passengers will be let out in an hour, the three then steal their clothes to get Billy and Moonface out in time to stop the wedding. On the deck, Erma is proposed to by all the sailors she's slept with during the cruise. She warns them if they start a relationship, she won't be easily pleased ("Buddy Beware").
+The wedding starts but is interrupted when Reno, Billy, and Moonface run in wearing Chinese garb. They claim that Reno is Plum Blossom, who is actually a Chinese princess that Evelyn dishonored when he slept with her. The ruse is almost ruined when Moonface accepts Eli's bribe to leave, but Hope intervenes by saying the only way for Evelyn to right his wrong is if he offers her to Plum Blossom's relative. Evelyn goes along with this, giving Hope away to Billy, and then proposing to Reno who accepts as she unmasks herself. Evangeline is distraught over the idea of becoming poor, but Eli proposes to her, bragging that his recent Wall Street sale has made him rich. Their mutual delight is cut short when Billy unveils his identity and informs his boss that he never made the sale. Evangeline prepares to leave Eli immediately but before she can do so, a wire comes in saying that the stock that wasn't sold has gone through the roof making him even richer than he imagined. All three couples now together sing to each other as they're married and the whole ship celebrates ("Finale").</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">

</xml_diff>